<commit_message>
Sincronizacion: Ordenamiento Gantt por Nivel Planificacion, ajuste de etiquetas en tooltip y diagnostico de anomalias en Proyecto 25-063
</commit_message>
<xml_diff>
--- a/Excel Planificacion/plif..xlsx
+++ b/Excel Planificacion/plif..xlsx
@@ -1,21 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistemas ABBAMAT\planificacionProcesosProductivos EN DESARROLLO\Excel Planificacion\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="Hoja1"/>
-    <sheet r:id="rId2" sheetId="2" name="Hoja2"/>
+    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="152511"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="32">
   <si>
     <t>QUE QUEREMOS VER</t>
   </si>
@@ -92,6 +97,9 @@
     <t>mejorar filtrado de proyecto (ver papel 1)</t>
   </si>
   <si>
+    <t>LO MISMO QUE LA FILA DE ARRIBA</t>
+  </si>
+  <si>
     <t>la maquina debe cambiarse con un desplegable(no arrastrar)</t>
   </si>
   <si>
@@ -99,17 +107,22 @@
   </si>
   <si>
     <t>por que cambia de color al tocar una celda?</t>
+  </si>
+  <si>
+    <t>PARA DARSE CUENTA QUE ESE VALOR NO ES EL ORIGINAL DEL EQUAL. QUE ALGUIEN LO MODIFICÓ</t>
   </si>
   <si>
     <t>factor de eficiencia????mmm
 me suena a IA</t>
+  </si>
+  <si>
+    <t>HAY QUE VER COMO SE IMPLEMENTA, NO TODAS LAS DENOMINACIONES TIENEN ARTICULO ( Hay que estandarizar como se representa el ARTICULO dentro de la DENOMINACION )</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -120,7 +133,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9c0006"/>
+      <color rgb="FF9C0006"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -146,12 +159,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFffc7ce"/>
+        <fgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFc6efce"/>
+        <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -165,16 +178,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </left>
       <right style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </right>
       <top style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </bottom>
       <diagonal/>
     </border>
@@ -190,52 +203,51 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="13">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -246,10 +258,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -287,71 +299,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -379,7 +391,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -402,11 +414,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -415,13 +427,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -431,7 +443,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -440,7 +452,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -449,7 +461,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -457,10 +469,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -530,24 +542,14 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:M30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="10" width="27.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="11" width="35.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="27.7109375" style="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.5703125" style="11" customWidth="1"/>
+    <col min="3" max="13" width="13.5703125" style="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
+    <row r="1" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -566,7 +568,7 @@
       <c r="L1" s="4"/>
       <c r="M1" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row r="2" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>2</v>
       </c>
@@ -585,7 +587,7 @@
       <c r="L2" s="3"/>
       <c r="M2" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row r="3" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>4</v>
       </c>
@@ -604,7 +606,7 @@
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row r="4" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>6</v>
       </c>
@@ -623,7 +625,7 @@
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row r="5" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>8</v>
       </c>
@@ -642,7 +644,7 @@
       <c r="L5" s="3"/>
       <c r="M5" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="31.5">
+    <row r="6" spans="1:13" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>10</v>
       </c>
@@ -661,7 +663,7 @@
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    <row r="7" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
       <c r="B7" s="5" t="s">
         <v>12</v>
@@ -678,7 +680,7 @@
       <c r="L7" s="3"/>
       <c r="M7" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+    <row r="8" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5"/>
       <c r="B8" s="5" t="s">
         <v>13</v>
@@ -695,7 +697,7 @@
       <c r="L8" s="3"/>
       <c r="M8" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+    <row r="9" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5"/>
       <c r="B9" s="5" t="s">
         <v>14</v>
@@ -712,7 +714,7 @@
       <c r="L9" s="3"/>
       <c r="M9" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+    <row r="10" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5"/>
       <c r="B10" s="5" t="s">
         <v>15</v>
@@ -729,7 +731,7 @@
       <c r="L10" s="3"/>
       <c r="M10" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+    <row r="11" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5"/>
       <c r="B11" s="5" t="s">
         <v>16</v>
@@ -746,7 +748,7 @@
       <c r="L11" s="3"/>
       <c r="M11" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+    <row r="12" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="6"/>
@@ -761,7 +763,7 @@
       <c r="L12" s="3"/>
       <c r="M12" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+    <row r="13" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7"/>
       <c r="B13" s="8"/>
       <c r="C13" s="6"/>
@@ -776,7 +778,7 @@
       <c r="L13" s="3"/>
       <c r="M13" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+    <row r="14" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="7"/>
       <c r="B14" s="8"/>
       <c r="C14" s="6"/>
@@ -791,7 +793,7 @@
       <c r="L14" s="3"/>
       <c r="M14" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+    <row r="15" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7"/>
       <c r="B15" s="8"/>
       <c r="C15" s="6"/>
@@ -806,7 +808,7 @@
       <c r="L15" s="3"/>
       <c r="M15" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+    <row r="16" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="7"/>
       <c r="B16" s="8"/>
       <c r="C16" s="6"/>
@@ -821,7 +823,7 @@
       <c r="L16" s="3"/>
       <c r="M16" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+    <row r="17" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="7"/>
       <c r="B17" s="8"/>
       <c r="C17" s="6"/>
@@ -836,7 +838,7 @@
       <c r="L17" s="3"/>
       <c r="M17" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
+    <row r="18" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="7"/>
       <c r="B18" s="8"/>
       <c r="C18" s="6"/>
@@ -851,7 +853,7 @@
       <c r="L18" s="3"/>
       <c r="M18" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
+    <row r="19" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>17</v>
       </c>
@@ -868,7 +870,7 @@
       <c r="L19" s="3"/>
       <c r="M19" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
+    <row r="20" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>18</v>
       </c>
@@ -887,7 +889,7 @@
       <c r="L20" s="3"/>
       <c r="M20" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="31.5">
+    <row r="21" spans="1:13" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>20</v>
       </c>
@@ -906,11 +908,13 @@
       <c r="L21" s="3"/>
       <c r="M21" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="31.5">
+    <row r="22" spans="1:13" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B22" s="8"/>
+      <c r="B22" s="8" t="s">
+        <v>19</v>
+      </c>
       <c r="C22" s="6"/>
       <c r="D22" s="6"/>
       <c r="E22" s="6"/>
@@ -923,11 +927,13 @@
       <c r="L22" s="3"/>
       <c r="M22" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
+    <row r="23" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="8"/>
+      <c r="B23" s="8" t="s">
+        <v>19</v>
+      </c>
       <c r="C23" s="6"/>
       <c r="D23" s="6"/>
       <c r="E23" s="6"/>
@@ -940,11 +946,13 @@
       <c r="L23" s="3"/>
       <c r="M23" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="44.25">
+    <row r="24" spans="1:13" ht="87" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B24" s="8"/>
+      <c r="B24" s="8" t="s">
+        <v>31</v>
+      </c>
       <c r="C24" s="6"/>
       <c r="D24" s="6"/>
       <c r="E24" s="6"/>
@@ -957,11 +965,13 @@
       <c r="L24" s="3"/>
       <c r="M24" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="31.5">
+    <row r="25" spans="1:13" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B25" s="8"/>
+      <c r="B25" s="8" t="s">
+        <v>25</v>
+      </c>
       <c r="C25" s="6"/>
       <c r="D25" s="6"/>
       <c r="E25" s="6"/>
@@ -974,11 +984,13 @@
       <c r="L25" s="3"/>
       <c r="M25" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="44.25">
+    <row r="26" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B26" s="8"/>
+        <v>26</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>19</v>
+      </c>
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
       <c r="E26" s="6"/>
@@ -991,11 +1003,13 @@
       <c r="L26" s="3"/>
       <c r="M26" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="31.5">
+    <row r="27" spans="1:13" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B27" s="8"/>
+        <v>27</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>19</v>
+      </c>
       <c r="C27" s="6"/>
       <c r="D27" s="6"/>
       <c r="E27" s="6"/>
@@ -1008,11 +1022,13 @@
       <c r="L27" s="3"/>
       <c r="M27" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="31.5">
+    <row r="28" spans="1:13" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B28" s="8"/>
+        <v>28</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>29</v>
+      </c>
       <c r="C28" s="6"/>
       <c r="D28" s="6"/>
       <c r="E28" s="6"/>
@@ -1025,9 +1041,9 @@
       <c r="L28" s="3"/>
       <c r="M28" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="31.5">
+    <row r="29" spans="1:13" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B29" s="8"/>
       <c r="C29" s="6"/>
@@ -1042,7 +1058,7 @@
       <c r="L29" s="3"/>
       <c r="M29" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
+    <row r="30" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="6"/>
       <c r="B30" s="8"/>
       <c r="C30" s="3"/>
@@ -1068,7 +1084,7 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>